<commit_message>
Change validation logic: No = blank, blank = pass through data
Flip the convention so you only mark fields "No" to blank them out.
Leave cells empty in the Excel to pass through whatever data exists.
This is simpler — you only fill in the cells you want to suppress.

https://claude.ai/code/session_01JA9wAKoEn1hihmhgHjy4Ab
</commit_message>
<xml_diff>
--- a/config/program_validation.xlsx
+++ b/config/program_validation.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>VA Suicide Prevention — no SSVF fields</t>
+          <t>VA Suicide Prevention — blank all fields</t>
         </is>
       </c>
     </row>
@@ -541,19 +541,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>SHIP program — RRH so Housed applies, has Legal</t>
+          <t>SHIP RRH — Legal and Housed pull through</t>
         </is>
       </c>
     </row>
@@ -600,7 +592,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>CDBG program</t>
+          <t>CDBG — blank all fields</t>
         </is>
       </c>
     </row>
@@ -635,19 +627,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>All EHA programs</t>
+          <t>All EHA programs — Legal and Housed pull through</t>
         </is>
       </c>
     </row>

</xml_diff>